<commit_message>
fix small details such as download template
</commit_message>
<xml_diff>
--- a/data/oecd_comments.xlsx
+++ b/data/oecd_comments.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Kate/OneDrive/WISE/Data request portal/data-request-portal/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B09990E4-C437-9945-863D-F5ACC17B3CA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4D81FB9-3833-E94B-9194-374385804112}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,15 @@
     <sheet name="Sheet 1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet 1'!$A$1:$C$61</definedName>
+  </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="65">
   <si>
     <t>ref_area</t>
   </si>
@@ -41,24 +44,18 @@
     <t>1_5</t>
   </si>
   <si>
-    <t>Metadata was previously filled out, but no data was provided due to non-conformity of question formats.</t>
-  </si>
-  <si>
-    <t>Data was flagged as available in latest questionnaire, but was not entered.</t>
-  </si>
-  <si>
     <t>4_1</t>
   </si>
   <si>
+    <t>4_2</t>
+  </si>
+  <si>
     <t>4_3</t>
   </si>
   <si>
     <t>5_5</t>
   </si>
   <si>
-    <t>Data was entered in previous request, but were not comparable. Please validate previous responses and enter the values again.</t>
-  </si>
-  <si>
     <t>7_2</t>
   </si>
   <si>
@@ -68,15 +65,176 @@
     <t>BEL</t>
   </si>
   <si>
-    <t>Different values were provided in the 2022 and 2025 questionnaires, the 2025 version is currently being used. Please validate the data and confirm it corresponds with Belgium's statistics.</t>
+    <t>CAN</t>
+  </si>
+  <si>
+    <t>9_1</t>
+  </si>
+  <si>
+    <t>14_1</t>
+  </si>
+  <si>
+    <t>14_2</t>
+  </si>
+  <si>
+    <t>COL</t>
+  </si>
+  <si>
+    <t>7_3</t>
+  </si>
+  <si>
+    <t>7_4</t>
+  </si>
+  <si>
+    <t>CRI</t>
+  </si>
+  <si>
+    <t>EST</t>
+  </si>
+  <si>
+    <t>GRC</t>
+  </si>
+  <si>
+    <t>Different values were provided in the 2022 and 2025 questionnaires. We are currently using the 2025 version - please validate the values below and confirm they align with Belgium's official statistics.</t>
+  </si>
+  <si>
+    <t>Thank you for submitting data in a previous request. Unfortunately we were not able to harmonize it with the other data in the Well-being Database due to incomplete information on the Time Use data. To remedy this, please fill out the Time Use Tables on the Time Use Submission page so we may validate the data.</t>
+  </si>
+  <si>
+    <t>ISR</t>
+  </si>
+  <si>
+    <t>2_9</t>
+  </si>
+  <si>
+    <t>reason</t>
+  </si>
+  <si>
+    <t>MEX</t>
+  </si>
+  <si>
+    <t>5-point scale rather than 6-point used by the OECD</t>
+  </si>
+  <si>
+    <t>CES-D-7 is not directly comparable to PHQ-8/9</t>
+  </si>
+  <si>
+    <t>Data only covers population 50 years and older</t>
+  </si>
+  <si>
+    <t>NZL</t>
+  </si>
+  <si>
+    <t>4-point scale rather than 6-point used by the OECD</t>
+  </si>
+  <si>
+    <t>3_5</t>
+  </si>
+  <si>
+    <t>4-point scale rather than yes/no used by the OECD</t>
+  </si>
+  <si>
+    <t>4_4</t>
+  </si>
+  <si>
+    <t>3-point scale rather than 11-point scale used by the OECD</t>
+  </si>
+  <si>
+    <t>NOR</t>
+  </si>
+  <si>
+    <t>Thank you for sharing this data. In the previous request, the country average was not included among the data shared, would you it be possible to update the values to include it?</t>
+  </si>
+  <si>
+    <t>POL</t>
+  </si>
+  <si>
+    <t>KOR</t>
+  </si>
+  <si>
+    <t>4-point scale rather than 11-point scale used by the OECD</t>
+  </si>
+  <si>
+    <t>5-point scale rather than 11-point scale used by the OECD</t>
+  </si>
+  <si>
+    <t>4-point scale rather than 5-point scale used by the OECD</t>
+  </si>
+  <si>
+    <t>Thank you for letting us know about this indicator in previous data submissions. Unfortunately, it doesn't match the OECD response format, so we're unable to publish it in the Well-being Database. We're still happy to receive any updated submissions on it for record-keeping, where it remains available for future reference and analysis.</t>
+  </si>
+  <si>
+    <t>Thank you for submitting this data. However in the previous submission, the metadata shared refers to anxiety and not depresssion. Could you verify if data related to depressive symptoms are available?</t>
+  </si>
+  <si>
+    <t>4-point scale rather than 10-point scale used by the OECD</t>
+  </si>
+  <si>
+    <t>CHE</t>
+  </si>
+  <si>
+    <t>TUR</t>
+  </si>
+  <si>
+    <t>GBR</t>
+  </si>
+  <si>
+    <t>5-point scale rather than 10-point scale used by the OECD</t>
+  </si>
+  <si>
+    <t>5-point scale rather than 10-point scale used by the OECD. EU-SILC data is currently being used.</t>
+  </si>
+  <si>
+    <t>7-point scale rather than 10-point scale used by the OECD. EU-SILC data is currently being used.</t>
+  </si>
+  <si>
+    <t>USA</t>
+  </si>
+  <si>
+    <t>11_1</t>
+  </si>
+  <si>
+    <t>Question phrasing is different from OECD's source.</t>
+  </si>
+  <si>
+    <t>Data was flagged as available in latest questionnaire, but was not provided. We would be happy to accept the data if it is available.</t>
+  </si>
+  <si>
+    <t>Data was provided in previous request, but this indicator is under review in our Well-being Framework so methodology validation is pending. We're still happy to accept data updates so that it may be available for integration in the future.</t>
+  </si>
+  <si>
+    <t>Collected by non-offical source (Scanlon Institute)</t>
+  </si>
+  <si>
+    <t>2-point scale rather than 10-point scale used by the OECD</t>
+  </si>
+  <si>
+    <t>5-point scale rather than 6-point scale used by the OECD</t>
+  </si>
+  <si>
+    <t>2-point scale rather than 5-point scale used by the OECD</t>
+  </si>
+  <si>
+    <t>4-point scale rather than 6-point scale used by the OECD</t>
+  </si>
+  <si>
+    <t>Thank you for submitting data in a previous request. However the percentages should be in percentage of the subgroup (so number of women who voted / percentage of total population of women) not the entire population. Would it be possible to provide data by subgroup?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -104,9 +262,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -405,24 +567,29 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C9"/>
+  <sheetPr filterMode="1"/>
+  <dimension ref="A1:D61"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="51.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="65.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="27.1640625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+      <c r="D1" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>3</v>
       </c>
@@ -430,32 +597,35 @@
         <v>5</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+        <v>45</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
       <c r="B3" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="64" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -463,54 +633,715 @@
         <v>4</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>3</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="64" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>3</v>
       </c>
       <c r="B7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="32" x14ac:dyDescent="0.2">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>3</v>
       </c>
       <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A10" t="s">
         <v>13</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="B10" t="s">
+        <v>15</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>16</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A12" t="s">
+        <v>13</v>
+      </c>
+      <c r="B12" t="s">
+        <v>4</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B13" t="s">
+        <v>9</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A14" t="s">
+        <v>13</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A15" t="s">
+        <v>13</v>
+      </c>
+      <c r="B15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A16" t="s">
+        <v>17</v>
+      </c>
+      <c r="B16" t="s">
+        <v>6</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A17" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="64" x14ac:dyDescent="0.2">
-      <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="C17" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A18" t="s">
+        <v>17</v>
+      </c>
+      <c r="B18" t="s">
+        <v>8</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A19" t="s">
+        <v>17</v>
+      </c>
+      <c r="B19" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A20" t="s">
+        <v>17</v>
+      </c>
+      <c r="B20" t="s">
+        <v>18</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A21" t="s">
+        <v>17</v>
+      </c>
+      <c r="B21" t="s">
+        <v>19</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A22" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>6</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A23" t="s">
+        <v>20</v>
+      </c>
+      <c r="B23" t="s">
+        <v>7</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A24" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A25" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C25" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A26" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A27" t="s">
+        <v>21</v>
+      </c>
+      <c r="B27" t="s">
+        <v>6</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A28" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" t="s">
+        <v>10</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A29" t="s">
+        <v>22</v>
+      </c>
+      <c r="B29" t="s">
+        <v>7</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A30" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A31" t="s">
+        <v>25</v>
+      </c>
+      <c r="B31" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A32" t="s">
+        <v>28</v>
+      </c>
+      <c r="B32" t="s">
+        <v>5</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A33" t="s">
+        <v>28</v>
+      </c>
+      <c r="B33" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A34" t="s">
+        <v>28</v>
+      </c>
+      <c r="B34" t="s">
+        <v>19</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A35" t="s">
+        <v>32</v>
+      </c>
+      <c r="B35" t="s">
+        <v>5</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A36" t="s">
+        <v>32</v>
+      </c>
+      <c r="B36" t="s">
+        <v>26</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A37" t="s">
+        <v>32</v>
+      </c>
+      <c r="B37" t="s">
+        <v>34</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A38" t="s">
+        <v>32</v>
+      </c>
+      <c r="B38" t="s">
+        <v>36</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A39" t="s">
+        <v>38</v>
+      </c>
+      <c r="B39" t="s">
+        <v>16</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A40" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" t="s">
+        <v>6</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A41" t="s">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A42" t="s">
+        <v>41</v>
+      </c>
+      <c r="B42" t="s">
+        <v>6</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A43" t="s">
+        <v>41</v>
+      </c>
+      <c r="B43" t="s">
+        <v>8</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A44" t="s">
+        <v>41</v>
+      </c>
+      <c r="B44" t="s">
+        <v>36</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A45" t="s">
+        <v>41</v>
+      </c>
+      <c r="B45" t="s">
+        <v>4</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A46" t="s">
+        <v>41</v>
+      </c>
+      <c r="B46" t="s">
+        <v>18</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A47" t="s">
+        <v>41</v>
+      </c>
+      <c r="B47" t="s">
+        <v>19</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A48" t="s">
+        <v>41</v>
+      </c>
+      <c r="B48" t="s">
         <v>15</v>
       </c>
+      <c r="C48" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A49" t="s">
+        <v>41</v>
+      </c>
+      <c r="B49" t="s">
+        <v>16</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A50" t="s">
+        <v>48</v>
+      </c>
+      <c r="B50" t="s">
+        <v>7</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A51" t="s">
+        <v>48</v>
+      </c>
+      <c r="B51" t="s">
+        <v>8</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" ht="48" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A52" t="s">
+        <v>48</v>
+      </c>
+      <c r="B52" t="s">
+        <v>9</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" ht="64" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A53" t="s">
+        <v>49</v>
+      </c>
+      <c r="B53" t="s">
+        <v>11</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A54" t="s">
+        <v>50</v>
+      </c>
+      <c r="B54" t="s">
+        <v>26</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" ht="32" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A55" t="s">
+        <v>50</v>
+      </c>
+      <c r="B55" t="s">
+        <v>34</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A56" t="s">
+        <v>50</v>
+      </c>
+      <c r="B56" t="s">
+        <v>36</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A57" t="s">
+        <v>50</v>
+      </c>
+      <c r="B57" t="s">
+        <v>18</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A58" t="s">
+        <v>54</v>
+      </c>
+      <c r="B58" t="s">
+        <v>6</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A59" t="s">
+        <v>54</v>
+      </c>
+      <c r="B59" t="s">
+        <v>8</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" ht="64" x14ac:dyDescent="0.2">
+      <c r="A60" t="s">
+        <v>54</v>
+      </c>
+      <c r="B60" t="s">
+        <v>10</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" ht="80" hidden="1" x14ac:dyDescent="0.2">
+      <c r="A61" t="s">
+        <v>54</v>
+      </c>
+      <c r="B61" t="s">
+        <v>55</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>56</v>
+      </c>
     </row>
   </sheetData>
+  <autoFilter xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" ref="A1:C61" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="2">
+      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice Requires="x14">
+          <filters>
+            <x14:filter val="Thank you for submitting data in a previous request. Unfortunately we were not able to harmonize it with the other data in the Well-being Database due to incomplete information on the Time Use data. To remedy this, please fill out the Time Use Tables on the Time Use Submission page so we may validate the data."/>
+          </filters>
+        </mc:Choice>
+        <mc:Fallback>
+          <customFilters>
+            <customFilter val=""/>
+            <customFilter operator="notEqual" val=" "/>
+          </customFilters>
+        </mc:Fallback>
+      </mc:AlternateContent>
+    </filterColumn>
+  </autoFilter>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C29">
+    <sortCondition ref="A1:A29"/>
+  </sortState>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>

</xml_diff>